<commit_message>
Add Dockerfile and model
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,87 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>45762.5139752438</v>
+        <v>45762.51397524306</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dinesh</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dineshkumarpolavarapu5@gmail.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pbkdf2:sha256:260000$JdA1MFdO7V3D3UKa$a46f6aa26a68dd6e580cc9c7a74ef78c26b346574a3ad06235ecd1e3356849f6</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>45771.72342819445</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Aarthi</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>aarthi@datapro.in</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$BkAgABPSrPXREsqT$ac445a4b7af17334590e90d527effe74b002d70516785257d39aa73c293185186acb17c921a5e346954c26ca88737f78ceee2878475ebf17d6fe8036dcf856b5</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>45856.18787439815</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Upendra</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>alekhya121@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$WOZTP6oDm6qYcbs3$54fa72c5ba613ad3385fc17b36586d8b1c0feb8c18fc63e39225e34e0551a69572d7b5dfb996c4e0a7c6a535749baf88cd0afd84d78f575b1a778afe61038ef0</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>45881.48849262732</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>vinay</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>vinay25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$ba7lZxGf666p2g7G$cb25a430dc8288cdc01dda71c51414c4d084c0b6ccde0316cfd0345a6dab5d5ddf5059ab4937c121f12a89c41d40a96ced841374416b05393066c2cc7a74bf8f</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>45887.49879161496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>